<commit_message>
Texture cache and skybox
</commit_message>
<xml_diff>
--- a/P3DBenchmark/Performance.xlsx
+++ b/P3DBenchmark/Performance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\Potato3d\P3DBenchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E41BDA-6D04-4957-9DF2-EAE5E8F362F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A33BB3-D0B9-4F4E-A122-CD9E1A47F506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{86B0D043-EEC2-43D0-BCB6-CB5E79D6E46A}"/>
+    <workbookView xWindow="180" yWindow="6555" windowWidth="20820" windowHeight="8385" xr2:uid="{86B0D043-EEC2-43D0-BCB6-CB5E79D6E46A}"/>
   </bookViews>
   <sheets>
     <sheet name="Tex, Flags&lt;0&gt;" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="73">
   <si>
     <t>GCC Win</t>
   </si>
@@ -245,6 +245,12 @@
   </si>
   <si>
     <t>Edge Refactor</t>
+  </si>
+  <si>
+    <t>Unsigned int UV</t>
+  </si>
+  <si>
+    <t>Texture cache</t>
   </si>
 </sst>
 </file>
@@ -663,11 +669,11 @@
         <v>76</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E5" si="0">(D3/D$2)-1</f>
+        <f>(D3/D$2)-1</f>
         <v>0.35714285714285721</v>
       </c>
       <c r="F3" s="1">
-        <f t="shared" ref="F3:F34" si="1">(D3/D2)-1</f>
+        <f t="shared" ref="F3:F36" si="0">(D3/D2)-1</f>
         <v>0.35714285714285721</v>
       </c>
     </row>
@@ -685,11 +691,11 @@
         <v>75</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" si="0"/>
+        <f>(D4/D$2)-1</f>
         <v>0.33928571428571419</v>
       </c>
       <c r="F4" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-1.3157894736842146E-2</v>
       </c>
       <c r="H4">
@@ -710,11 +716,11 @@
         <v>75</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E3:E5" si="1">(D5/D$2)-1</f>
         <v>0.33928571428571419</v>
       </c>
       <c r="F5" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H5">
@@ -739,7 +745,7 @@
         <v>0.33928571428571419</v>
       </c>
       <c r="F6" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H6">
@@ -764,7 +770,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.12000000000000011</v>
       </c>
       <c r="H7">
@@ -789,7 +795,7 @@
         <v>0.48214285714285721</v>
       </c>
       <c r="F8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-1.1904761904761862E-2</v>
       </c>
       <c r="H8">
@@ -814,7 +820,7 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="F9" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>6.024096385542177E-2</v>
       </c>
     </row>
@@ -836,7 +842,7 @@
         <v>0.60714285714285721</v>
       </c>
       <c r="F10" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.2727272727272707E-2</v>
       </c>
       <c r="H10">
@@ -855,7 +861,7 @@
         <v>0.64285714285714279</v>
       </c>
       <c r="F11" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.2222222222222143E-2</v>
       </c>
     </row>
@@ -877,7 +883,7 @@
         <v>0.75</v>
       </c>
       <c r="F12" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>6.5217391304347894E-2</v>
       </c>
     </row>
@@ -899,7 +905,7 @@
         <v>0.75</v>
       </c>
       <c r="F13" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H13">
@@ -924,7 +930,7 @@
         <v>0.76785714285714279</v>
       </c>
       <c r="F14" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.0204081632652962E-2</v>
       </c>
     </row>
@@ -942,11 +948,11 @@
         <v>115</v>
       </c>
       <c r="E15" s="1">
-        <f t="shared" ref="E15:E34" si="3">(D15/D$2)-1</f>
+        <f t="shared" ref="E15:E36" si="3">(D15/D$2)-1</f>
         <v>1.0535714285714284</v>
       </c>
       <c r="F15" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.16161616161616155</v>
       </c>
     </row>
@@ -968,7 +974,7 @@
         <v>1.0357142857142856</v>
       </c>
       <c r="F16" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-8.6956521739129933E-3</v>
       </c>
       <c r="H16">
@@ -993,7 +999,7 @@
         <v>1.0357142857142856</v>
       </c>
       <c r="F17" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H17">
@@ -1018,7 +1024,7 @@
         <v>1.0357142857142856</v>
       </c>
       <c r="F18" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H18">
@@ -1043,7 +1049,7 @@
         <v>1.0357142857142856</v>
       </c>
       <c r="F19" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H19">
@@ -1068,7 +1074,7 @@
         <v>1.0714285714285716</v>
       </c>
       <c r="F20" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.7543859649122862E-2</v>
       </c>
       <c r="H20">
@@ -1093,7 +1099,7 @@
         <v>1.0714285714285716</v>
       </c>
       <c r="F21" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H21">
@@ -1118,7 +1124,7 @@
         <v>1.0714285714285716</v>
       </c>
       <c r="F22" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H22">
@@ -1143,7 +1149,7 @@
         <v>0.96428571428571419</v>
       </c>
       <c r="F23" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-5.1724137931034475E-2</v>
       </c>
       <c r="H23">
@@ -1162,7 +1168,7 @@
         <v>1.1964285714285716</v>
       </c>
       <c r="F24" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.11818181818181817</v>
       </c>
       <c r="H24">
@@ -1187,7 +1193,7 @@
         <v>1.0357142857142856</v>
       </c>
       <c r="F25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-7.3170731707317027E-2</v>
       </c>
       <c r="H25">
@@ -1212,7 +1218,7 @@
         <v>1.0357142857142856</v>
       </c>
       <c r="F26" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H26">
@@ -1231,7 +1237,7 @@
         <v>0.96428571428571419</v>
       </c>
       <c r="F27" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-3.5087719298245612E-2</v>
       </c>
     </row>
@@ -1247,7 +1253,7 @@
         <v>1.0892857142857144</v>
       </c>
       <c r="F28" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>6.3636363636363713E-2</v>
       </c>
       <c r="H28">
@@ -1266,7 +1272,7 @@
         <v>0.96428571428571419</v>
       </c>
       <c r="F29" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-5.9829059829059839E-2</v>
       </c>
     </row>
@@ -1282,7 +1288,7 @@
         <v>1.0535714285714284</v>
       </c>
       <c r="F30" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.5454545454545414E-2</v>
       </c>
       <c r="H30">
@@ -1301,7 +1307,7 @@
         <v>0.9464285714285714</v>
       </c>
       <c r="F31" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-5.2173913043478293E-2</v>
       </c>
     </row>
@@ -1317,7 +1323,7 @@
         <v>1.1785714285714284</v>
       </c>
       <c r="F32" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.11926605504587151</v>
       </c>
     </row>
@@ -1333,7 +1339,7 @@
         <v>0.9464285714285714</v>
       </c>
       <c r="F33" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-0.10655737704918034</v>
       </c>
     </row>
@@ -1349,8 +1355,40 @@
         <v>1.0892857142857144</v>
       </c>
       <c r="F34" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>7.3394495412844041E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="2">
+        <v>120</v>
+      </c>
+      <c r="E35" s="1">
+        <f t="shared" si="3"/>
+        <v>1.1428571428571428</v>
+      </c>
+      <c r="F35" s="1">
+        <f t="shared" si="0"/>
+        <v>2.564102564102555E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="2">
+        <v>137</v>
+      </c>
+      <c r="E36" s="1">
+        <f t="shared" si="3"/>
+        <v>1.4464285714285716</v>
+      </c>
+      <c r="F36" s="1">
+        <f t="shared" si="0"/>
+        <v>0.14166666666666661</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1418,7 +1456,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4F0AC41-34A4-4C4B-992F-CC4F79B64425}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
@@ -1472,11 +1510,11 @@
         <v>248</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E27" si="0">(D3/D$2)-1</f>
+        <f t="shared" ref="E3:E28" si="0">(D3/D$2)-1</f>
         <v>-0.3737373737373737</v>
       </c>
       <c r="F3" s="1">
-        <f t="shared" ref="F3:F27" si="1">(D3/D2)-1</f>
+        <f t="shared" ref="F3:F28" si="1">(D3/D2)-1</f>
         <v>-0.3737373737373737</v>
       </c>
     </row>
@@ -1976,6 +2014,22 @@
       <c r="F27" s="1">
         <f t="shared" si="1"/>
         <v>3.2064128256513058E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28">
+        <v>501</v>
+      </c>
+      <c r="E28" s="1">
+        <f t="shared" si="0"/>
+        <v>0.26515151515151514</v>
+      </c>
+      <c r="F28" s="1">
+        <f t="shared" si="1"/>
+        <v>-2.7184466019417486E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2984,7 +3038,7 @@
         <v>98444</v>
       </c>
       <c r="D2" s="2">
-        <v>117</v>
+        <v>137</v>
       </c>
       <c r="E2" s="1">
         <f>(D2/D$2)-1</f>
@@ -3010,11 +3064,11 @@
       </c>
       <c r="E3" s="1">
         <f>(D3/D$2)-1</f>
-        <v>-0.17948717948717952</v>
+        <v>-0.2992700729927007</v>
       </c>
       <c r="F3" s="1">
         <f t="shared" ref="F3" si="0">(D3/D2)-1</f>
-        <v>-0.17948717948717952</v>
+        <v>-0.2992700729927007</v>
       </c>
       <c r="H3">
         <v>15016</v>
@@ -3031,11 +3085,11 @@
         <v>253228</v>
       </c>
       <c r="D6">
-        <v>549</v>
+        <v>501</v>
       </c>
       <c r="E6" s="1">
         <f>(D6/D$2)-1</f>
-        <v>3.6923076923076925</v>
+        <v>2.6569343065693429</v>
       </c>
       <c r="F6" s="1"/>
     </row>
@@ -3058,7 +3112,7 @@
       </c>
       <c r="F7" s="1">
         <f>(D7/D6)-1</f>
-        <v>-0.46448087431693985</v>
+        <v>-0.41317365269461082</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -3076,7 +3130,7 @@
       </c>
       <c r="E9" s="1">
         <f>(D9/D$2)-1</f>
-        <v>-0.28205128205128205</v>
+        <v>-0.38686131386861311</v>
       </c>
       <c r="F9" s="1"/>
       <c r="H9">

</xml_diff>